<commit_message>
feat: ExcelGenerator Enum 생성기 확장
- Enum.xlsx 시트를 파싱해 byte 기반 enum 소스 생성(None/Max 센티널 포함)
- Roslyn(Microsoft.CodeAnalysis)으로 즉석 컴파일 후 멤버 존재 여부 검증
- 생성 소스를 Output/Code/Enum.cs로 출력하는 MakeEnumCode 추가
- CallerFilePath 기반 ResolvePath로 소스 위치 기준 경로 해석
- 데이터 테이블 파싱용 ExcelGenerator.cs 골격 추가
</commit_message>
<xml_diff>
--- a/Server/ExcelGenerator/Excel/Item.xlsx
+++ b/Server/ExcelGenerator/Excel/Item.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/serotina/workspace/Windows_simulator/Server/ExcelGenerator/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wlsdn\workspace\Windows_simulator\Server\ExcelGenerator\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E598D920-A234-3F46-963F-0A8B8EE22CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622801CF-6ED8-49DF-BE3F-5343EAE881C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17100" yWindow="680" windowWidth="17120" windowHeight="19780" xr2:uid="{8228D3F1-03DA-484B-82A7-C04DAA9D8ADA}"/>
+    <workbookView xWindow="8505" yWindow="4935" windowWidth="28800" windowHeight="15345" xr2:uid="{8228D3F1-03DA-484B-82A7-C04DAA9D8ADA}"/>
   </bookViews>
   <sheets>
     <sheet name="ItemTable" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
   <si>
     <t>//</t>
     <phoneticPr fontId="0" type="noConversion"/>
@@ -160,17 +159,21 @@
   </si>
   <si>
     <t>MaxStack</t>
+  </si>
+  <si>
+    <t>s</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -178,7 +181,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -187,7 +190,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -268,7 +278,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -284,9 +294,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -324,7 +334,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -430,7 +440,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -572,7 +582,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -581,15 +591,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C3A7FA8-A593-D04F-ABC7-DFA8B90401BE}">
   <dimension ref="A2:G28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
     <col min="4" max="5" width="13.6640625" customWidth="1"/>
     <col min="6" max="6" width="16.33203125" customWidth="1"/>
-    <col min="7" max="7" width="67.83203125" customWidth="1"/>
+    <col min="7" max="7" width="67.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -612,7 +622,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -635,7 +645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -658,7 +668,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -669,7 +679,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -680,7 +690,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -691,7 +701,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="2" t="s">
         <v>10</v>
@@ -712,7 +722,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="5">
         <v>1</v>
@@ -733,7 +743,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="5">
         <v>2</v>
@@ -754,7 +764,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="5">
         <v>3</v>
@@ -775,7 +785,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="5">
         <v>4</v>
@@ -796,7 +806,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="5">
         <v>5</v>
@@ -817,7 +827,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="5">
         <v>6</v>
@@ -838,16 +848,18 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
+      <c r="E15" s="7" t="s">
+        <v>37</v>
+      </c>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="6"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -856,7 +868,7 @@
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -865,7 +877,7 @@
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -874,7 +886,7 @@
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -883,7 +895,7 @@
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -892,7 +904,7 @@
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -901,7 +913,7 @@
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="6"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -910,7 +922,7 @@
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="6"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -919,7 +931,7 @@
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -928,7 +940,7 @@
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="6"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -937,7 +949,7 @@
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="6"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -946,7 +958,7 @@
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="6"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -955,7 +967,7 @@
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="6"/>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -965,6 +977,8 @@
       <c r="G28" s="7"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ExcelGenerator - Code, DataPacker Data - bytes 추가
커밋해놓고 DataPacket는 ExcelGenerator로 옮김
</commit_message>
<xml_diff>
--- a/Server/ExcelGenerator/Excel/Item.xlsx
+++ b/Server/ExcelGenerator/Excel/Item.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wlsdn\workspace\Windows_simulator\Server\ExcelGenerator\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622801CF-6ED8-49DF-BE3F-5343EAE881C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{478AC77F-4981-4066-A1C9-D544C33572EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8505" yWindow="4935" windowWidth="28800" windowHeight="15345" xr2:uid="{8228D3F1-03DA-484B-82A7-C04DAA9D8ADA}"/>
+    <workbookView xWindow="-25170" yWindow="3930" windowWidth="28800" windowHeight="15345" xr2:uid="{8228D3F1-03DA-484B-82A7-C04DAA9D8ADA}"/>
   </bookViews>
   <sheets>
     <sheet name="ItemTable" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
   <si>
     <t>//</t>
     <phoneticPr fontId="0" type="noConversion"/>
@@ -85,46 +85,24 @@
   </si>
   <si>
     <t>Military1</t>
-  </si>
-  <si>
-    <t>Military1</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>SkillType1</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
   <si>
     <t>Military2</t>
   </si>
   <si>
-    <t>SkillType2</t>
-  </si>
-  <si>
     <t>Military3</t>
   </si>
   <si>
-    <t>SkillType3</t>
-  </si>
-  <si>
     <t>Shaman1</t>
   </si>
   <si>
-    <t>SkillType4</t>
-  </si>
-  <si>
     <t>Shaman2</t>
   </si>
   <si>
-    <t>SkillType5</t>
-  </si>
-  <si>
     <t>Shaman3</t>
   </si>
   <si>
-    <t>SkillType6</t>
-  </si>
-  <si>
     <t>아이템 TID</t>
   </si>
   <si>
@@ -141,9 +119,6 @@
   </si>
   <si>
     <t>ItemType</t>
-  </si>
-  <si>
-    <t>SkillType1</t>
   </si>
   <si>
     <t>ItemRarity</t>
@@ -163,6 +138,42 @@
   <si>
     <t>s</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>A</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>B</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>D</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>E</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>F</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Farming</t>
+  </si>
+  <si>
+    <t>Logging</t>
+  </si>
+  <si>
+    <t>Misc</t>
+  </si>
+  <si>
+    <t>Common</t>
   </si>
 </sst>
 </file>
@@ -250,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -275,6 +286,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -604,22 +618,22 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -656,10 +670,10 @@
         <v>6</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>5</v>
@@ -710,16 +724,16 @@
         <v>11</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -728,19 +742,19 @@
         <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" t="s">
+        <v>39</v>
       </c>
       <c r="F9" s="5">
         <v>1000</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -749,19 +763,19 @@
         <v>2</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>16</v>
+        <v>31</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" t="s">
+        <v>39</v>
       </c>
       <c r="F10" s="5">
         <v>2000</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -770,19 +784,19 @@
         <v>3</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>18</v>
+        <v>32</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
       </c>
       <c r="F11" s="5">
         <v>3000</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -791,19 +805,19 @@
         <v>4</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>20</v>
+        <v>33</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>39</v>
       </c>
       <c r="F12" s="5">
         <v>100</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -812,19 +826,19 @@
         <v>5</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>22</v>
+        <v>34</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
       </c>
       <c r="F13" s="5">
         <v>200</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -833,19 +847,19 @@
         <v>6</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>24</v>
+        <v>35</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" t="s">
+        <v>39</v>
       </c>
       <c r="F14" s="5">
         <v>300</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -854,7 +868,7 @@
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>

</xml_diff>